<commit_message>
Update agent status handling to use agent_status_code_id
</commit_message>
<xml_diff>
--- a/Documents/AgentUpload.xlsx
+++ b/Documents/AgentUpload.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Navin K\Desktop\Delete Me\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HMS2\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9A492C-E69E-44AD-A123-339AFABCE702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet3!$A$1:$H$106</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1259,7 +1258,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
@@ -1293,7 +1292,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1303,6 +1302,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1334,7 +1339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1350,6 +1355,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1379,9 +1385,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1419,9 +1425,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1456,7 +1462,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1491,7 +1497,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1664,143 +1670,143 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:ED7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="6.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="6.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.54296875" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.1796875" style="4" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="20.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="20.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="10.453125" style="4" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="18" style="4" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="10" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="15.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="5.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="19.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="17.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="17.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="8.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="15.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="5.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="17.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="17.453125" style="4" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="20.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="34.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="17.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="14.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="13.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="8.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="18.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="4.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="27.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="22.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="20.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="20.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="34.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="17.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="14.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="13.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="8.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="18.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="4.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="27.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="22.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="20.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="57" max="57" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="11.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="23.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="20.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="14.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="11.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="23.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="20.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="17" style="4" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="22.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="14.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="18.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="16.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="69" max="70" width="18.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="23.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="22.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="18.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="17.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="16.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="10.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="16.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="17.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="13.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="81" max="83" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="8.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="22.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="14.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="18.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="10.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="16.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="69" max="70" width="18.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="23.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="22.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="18.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="17.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="16.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="10.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="16.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="17.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="13.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="81" max="83" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="8.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="85" max="85" width="9" style="4" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="9.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="28.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="16.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="9.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="9.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="28.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="16.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="9.1796875" style="4" bestFit="1" customWidth="1"/>
     <col min="91" max="91" width="14" style="4" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="15.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="15.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="93" max="93" width="26" style="4" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="17.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="17.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="17.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="17.1796875" style="4" bestFit="1" customWidth="1"/>
     <col min="96" max="96" width="28" style="4" bestFit="1" customWidth="1"/>
     <col min="97" max="97" width="12" style="4" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="15.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="26.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="17.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="19.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="15.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="26.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="17.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="19.54296875" style="4" bestFit="1" customWidth="1"/>
     <col min="102" max="102" width="23" style="4" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="18.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="20.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="14.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="18.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="12.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="16.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="19.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="15.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="18.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="20.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="14.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="18.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="12.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="16.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="19.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="15.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
     <col min="113" max="113" width="10" style="4" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="17.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="19.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="12.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="11.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="14.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="23.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="11.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="25.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="17.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="19.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="12.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="11.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="14.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="23.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="11.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="25.1796875" style="4" bestFit="1" customWidth="1"/>
     <col min="123" max="123" width="11" style="4" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="15.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="19.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="126" max="127" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="12.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="14.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="15.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="19.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="126" max="127" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="12.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="14.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="14.54296875" style="4" bestFit="1" customWidth="1"/>
     <col min="131" max="131" width="19" style="4" bestFit="1" customWidth="1"/>
     <col min="132" max="132" width="14" style="4" bestFit="1" customWidth="1"/>
     <col min="133" max="133" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="10.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="135" max="16384" width="8.88671875" style="4"/>
+    <col min="134" max="134" width="10.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="135" max="16384" width="8.90625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:134" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="e">
         <f>VLOOKUP(A3,Sheet2!$A$1:$A$135,1,FALSE)</f>
         <v>#N/A</v>
@@ -1845,13 +1851,13 @@
         <f>IFERROR(VLOOKUP(K3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>PreferredLanguage</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="4" t="s">
         <v>405</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="4" t="s">
         <v>405</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="N1" s="4" t="s">
         <v>405</v>
       </c>
       <c r="O1" s="4" t="str">
@@ -1998,7 +2004,7 @@
         <f>IFERROR(VLOOKUP(AX3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>UlipFlag</v>
       </c>
-      <c r="AY1" s="4" t="str">
+      <c r="AY1" s="11" t="str">
         <f>IFERROR(VLOOKUP(AY3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>TrainingGroupType</v>
       </c>
@@ -2010,7 +2016,7 @@
         <f>IFERROR(VLOOKUP(BA3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>RefresherTrainingCompleted</v>
       </c>
-      <c r="BB1" s="4" t="str">
+      <c r="BB1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BB3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>IsMigrated</v>
       </c>
@@ -2026,7 +2032,7 @@
         <f>IFERROR(VLOOKUP(BE3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>RegistrationDate</v>
       </c>
-      <c r="BF1" s="4" t="str">
+      <c r="BF1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BF3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>Vertical</v>
       </c>
@@ -2042,15 +2048,15 @@
         <f>IFERROR(VLOOKUP(BI3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>IC36TrngCompletionDate</v>
       </c>
-      <c r="BJ1" s="4" t="str">
+      <c r="BJ1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BJ3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>STrngCompletionDate</v>
       </c>
-      <c r="BK1" s="4" t="str">
+      <c r="BK1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BK3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>ConfirmationDate</v>
       </c>
-      <c r="BL1" s="4" t="str">
+      <c r="BL1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BL3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>FgRockStarTrainingDate</v>
       </c>
@@ -2066,55 +2072,55 @@
         <f>IFERROR(VLOOKUP(BO3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>HRDoj</v>
       </c>
-      <c r="BP1" s="4" t="str">
-        <f>IFERROR(VLOOKUP(BP3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
-        <v>FgValueTrngDate</v>
-      </c>
-      <c r="BQ1" s="4" t="str">
+      <c r="BP1" s="11" t="str">
+        <f ca="1">IFERROR(BN11VLOOKUP(BP3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
+        <v>Ignore Field</v>
+      </c>
+      <c r="BQ1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BQ3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>HSecPolicyTrngDate</v>
       </c>
-      <c r="BR1" s="4" t="str">
+      <c r="BR1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BR3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>ITSecPolicyTrngDate</v>
       </c>
-      <c r="BS1" s="4" t="str">
+      <c r="BS1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BS3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>NPSTrngCompletionDate</v>
       </c>
-      <c r="BT1" s="4" t="str">
+      <c r="BT1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BT3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>WhistleBlowerTrngDate</v>
       </c>
-      <c r="BU1" s="4" t="str">
+      <c r="BU1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BU3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>GovPolicyTrngDate</v>
       </c>
-      <c r="BV1" s="4" t="str">
+      <c r="BV1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BV3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>InductionTrngDate</v>
       </c>
-      <c r="BW1" s="4" t="str">
+      <c r="BW1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BW3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>LastWorkingDate</v>
       </c>
-      <c r="BX1" s="4" t="str">
+      <c r="BX1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BX3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>LicenseNo</v>
       </c>
-      <c r="BY1" s="4" t="str">
+      <c r="BY1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BY3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>LicenseType</v>
       </c>
-      <c r="BZ1" s="4" t="str">
+      <c r="BZ1" s="11" t="str">
         <f>IFERROR(VLOOKUP(BZ3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>LicenseIssueDate</v>
       </c>
-      <c r="CA1" s="4" t="str">
+      <c r="CA1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CA3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>LicenseExpiryDate</v>
       </c>
-      <c r="CB1" s="4" t="str">
+      <c r="CB1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CB3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>LicenseStatus</v>
       </c>
@@ -2142,7 +2148,7 @@
         <f>IFERROR(VLOOKUP(CH3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>Landmark</v>
       </c>
-      <c r="CI1" s="4" t="str">
+      <c r="CI1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CI3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>AgentClassDesc</v>
       </c>
@@ -2196,27 +2202,27 @@
       <c r="CV1" s="10" t="s">
         <v>405</v>
       </c>
-      <c r="CW1" s="4" t="str">
+      <c r="CW1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CW3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>AgentTypeCodeDesc</v>
       </c>
-      <c r="CX1" s="4" t="str">
+      <c r="CX1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CX3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>AgentSubTypeCodeDesc</v>
       </c>
-      <c r="CY1" s="4" t="str">
+      <c r="CY1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CY3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>CandidateTypeDesc</v>
       </c>
-      <c r="CZ1" s="4" t="str">
+      <c r="CZ1" s="11" t="str">
         <f>IFERROR(VLOOKUP(CZ3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>CommissionClassDesc</v>
       </c>
-      <c r="DA1" s="4" t="str">
+      <c r="DA1" s="11" t="str">
         <f>IFERROR(VLOOKUP(DA3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>AgentTypeDesc</v>
       </c>
-      <c r="DB1" s="4" t="str">
+      <c r="DB1" s="11" t="str">
         <f>IFERROR(VLOOKUP(DB3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>NomineeName</v>
       </c>
@@ -2296,7 +2302,7 @@
         <f>IFERROR(VLOOKUP(DU3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>ResidenceContactNo</v>
       </c>
-      <c r="DV1" s="4" t="str">
+      <c r="DV1" s="11" t="str">
         <f>IFERROR(VLOOKUP(DV3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>BloodGroup</v>
       </c>
@@ -2324,19 +2330,19 @@
         <f>IFERROR(VLOOKUP(EB3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>AnnualIncome</v>
       </c>
-      <c r="EC1" s="4" t="str">
+      <c r="EC1" s="11" t="str">
         <f>IFERROR(VLOOKUP(EC3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>WorkExpMonths</v>
       </c>
-      <c r="ED1" s="4" t="str">
+      <c r="ED1" s="11" t="str">
         <f>IFERROR(VLOOKUP(ED3,Sheet2!$A$1:$A$135,1,FALSE),"Ignore Field")</f>
         <v>BranchDesc</v>
       </c>
     </row>
-    <row r="2" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:134" x14ac:dyDescent="0.35">
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:134" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2740,7 +2746,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:134" x14ac:dyDescent="0.35">
       <c r="B4" s="4" t="s">
         <v>167</v>
       </c>
@@ -3114,7 +3120,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="5" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:134" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
         <v>168</v>
       </c>
@@ -3485,7 +3491,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="6" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:134" x14ac:dyDescent="0.35">
       <c r="B6" s="4" t="s">
         <v>169</v>
       </c>
@@ -3856,7 +3862,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="7" spans="1:134" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:134" x14ac:dyDescent="0.35">
       <c r="B7" s="4" t="s">
         <v>170</v>
       </c>
@@ -4240,16 +4246,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CD3912-3EDB-4529-AEC7-5259CD4DE152}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:H106"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>381</v>
       </c>
@@ -4275,7 +4281,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>276</v>
       </c>
@@ -4301,7 +4307,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>277</v>
       </c>
@@ -4327,7 +4333,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>278</v>
       </c>
@@ -4353,7 +4359,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>279</v>
       </c>
@@ -4379,7 +4385,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>280</v>
       </c>
@@ -4405,7 +4411,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>281</v>
       </c>
@@ -4431,7 +4437,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>282</v>
       </c>
@@ -4457,7 +4463,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>283</v>
       </c>
@@ -4483,7 +4489,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>284</v>
       </c>
@@ -4509,7 +4515,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>285</v>
       </c>
@@ -4535,7 +4541,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>286</v>
       </c>
@@ -4561,7 +4567,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>287</v>
       </c>
@@ -4587,7 +4593,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>288</v>
       </c>
@@ -4613,7 +4619,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>289</v>
       </c>
@@ -4639,7 +4645,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>290</v>
       </c>
@@ -4665,7 +4671,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>291</v>
       </c>
@@ -4691,7 +4697,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>292</v>
       </c>
@@ -4717,7 +4723,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>293</v>
       </c>
@@ -4743,7 +4749,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>294</v>
       </c>
@@ -4769,7 +4775,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>295</v>
       </c>
@@ -4795,7 +4801,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>296</v>
       </c>
@@ -4821,7 +4827,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>297</v>
       </c>
@@ -4847,7 +4853,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>298</v>
       </c>
@@ -4873,7 +4879,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>299</v>
       </c>
@@ -4899,7 +4905,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>300</v>
       </c>
@@ -4925,7 +4931,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>301</v>
       </c>
@@ -4951,7 +4957,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>302</v>
       </c>
@@ -4977,7 +4983,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>303</v>
       </c>
@@ -5003,7 +5009,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>304</v>
       </c>
@@ -5029,7 +5035,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>305</v>
       </c>
@@ -5055,7 +5061,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>306</v>
       </c>
@@ -5081,7 +5087,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>307</v>
       </c>
@@ -5107,7 +5113,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>308</v>
       </c>
@@ -5133,7 +5139,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>309</v>
       </c>
@@ -5159,7 +5165,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>310</v>
       </c>
@@ -5185,7 +5191,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>311</v>
       </c>
@@ -5211,7 +5217,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>312</v>
       </c>
@@ -5237,7 +5243,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>313</v>
       </c>
@@ -5263,7 +5269,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>314</v>
       </c>
@@ -5289,7 +5295,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>315</v>
       </c>
@@ -5315,7 +5321,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>316</v>
       </c>
@@ -5341,7 +5347,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>317</v>
       </c>
@@ -5367,7 +5373,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>318</v>
       </c>
@@ -5393,7 +5399,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>319</v>
       </c>
@@ -5419,7 +5425,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>320</v>
       </c>
@@ -5445,7 +5451,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>321</v>
       </c>
@@ -5471,7 +5477,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>322</v>
       </c>
@@ -5497,7 +5503,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>323</v>
       </c>
@@ -5523,7 +5529,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>324</v>
       </c>
@@ -5549,7 +5555,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>325</v>
       </c>
@@ -5575,7 +5581,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>326</v>
       </c>
@@ -5601,7 +5607,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>327</v>
       </c>
@@ -5627,7 +5633,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>328</v>
       </c>
@@ -5653,7 +5659,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>329</v>
       </c>
@@ -5679,7 +5685,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>330</v>
       </c>
@@ -5705,7 +5711,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>331</v>
       </c>
@@ -5731,7 +5737,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>332</v>
       </c>
@@ -5757,7 +5763,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>333</v>
       </c>
@@ -5783,7 +5789,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>334</v>
       </c>
@@ -5809,7 +5815,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>335</v>
       </c>
@@ -5835,7 +5841,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>336</v>
       </c>
@@ -5861,7 +5867,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>337</v>
       </c>
@@ -5887,7 +5893,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>338</v>
       </c>
@@ -5913,7 +5919,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>339</v>
       </c>
@@ -5939,7 +5945,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>340</v>
       </c>
@@ -5965,7 +5971,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>341</v>
       </c>
@@ -5991,7 +5997,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>342</v>
       </c>
@@ -6017,7 +6023,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>343</v>
       </c>
@@ -6043,7 +6049,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>344</v>
       </c>
@@ -6069,7 +6075,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>345</v>
       </c>
@@ -6095,7 +6101,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>346</v>
       </c>
@@ -6121,7 +6127,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>347</v>
       </c>
@@ -6147,7 +6153,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>348</v>
       </c>
@@ -6173,7 +6179,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>349</v>
       </c>
@@ -6199,7 +6205,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>350</v>
       </c>
@@ -6225,7 +6231,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>351</v>
       </c>
@@ -6251,7 +6257,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>352</v>
       </c>
@@ -6277,7 +6283,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>353</v>
       </c>
@@ -6303,7 +6309,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>354</v>
       </c>
@@ -6329,7 +6335,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>355</v>
       </c>
@@ -6355,7 +6361,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>356</v>
       </c>
@@ -6381,7 +6387,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>357</v>
       </c>
@@ -6407,7 +6413,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>358</v>
       </c>
@@ -6433,7 +6439,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>359</v>
       </c>
@@ -6459,7 +6465,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>360</v>
       </c>
@@ -6485,7 +6491,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>361</v>
       </c>
@@ -6511,7 +6517,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>362</v>
       </c>
@@ -6537,7 +6543,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>363</v>
       </c>
@@ -6563,7 +6569,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>364</v>
       </c>
@@ -6589,7 +6595,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>365</v>
       </c>
@@ -6615,7 +6621,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>366</v>
       </c>
@@ -6641,7 +6647,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>367</v>
       </c>
@@ -6667,7 +6673,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>368</v>
       </c>
@@ -6693,7 +6699,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>369</v>
       </c>
@@ -6719,7 +6725,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>370</v>
       </c>
@@ -6745,7 +6751,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>371</v>
       </c>
@@ -6771,7 +6777,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>372</v>
       </c>
@@ -6797,7 +6803,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>373</v>
       </c>
@@ -6823,7 +6829,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>374</v>
       </c>
@@ -6849,7 +6855,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>375</v>
       </c>
@@ -6875,7 +6881,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>376</v>
       </c>
@@ -6901,7 +6907,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>377</v>
       </c>
@@ -6927,7 +6933,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>378</v>
       </c>
@@ -6953,7 +6959,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>379</v>
       </c>
@@ -6979,7 +6985,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>380</v>
       </c>
@@ -7006,7 +7012,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H106" xr:uid="{F7CD3912-3EDB-4529-AEC7-5259CD4DE152}">
+  <autoFilter ref="A1:H106">
     <filterColumn colId="5">
       <filters>
         <filter val="FALSE"/>
@@ -7018,684 +7024,684 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E55BC870-3E98-4962-845B-011F2F60DAD4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A135"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>260</v>
       </c>

</xml_diff>